<commit_message>
check cli vs curl usage
</commit_message>
<xml_diff>
--- a/eval/visualization/outputs/data/model_skills_report.xlsx
+++ b/eval/visualization/outputs/data/model_skills_report.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="grok-code-fast-1" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="minimax-m2.5-free" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="fm_skill_trigger_rate" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="pinchtab_cli_usage" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1293" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="105">
   <si>
     <t>Domain</t>
   </si>
@@ -322,6 +323,15 @@
   </si>
   <si>
     <t>opencode_minimax-m2.5-free</t>
+  </si>
+  <si>
+    <t>Pinchtab Tests</t>
+  </si>
+  <si>
+    <t>CLI Usage Tool Calls</t>
+  </si>
+  <si>
+    <t>curl.exe Usage Tool Calls</t>
   </si>
 </sst>
 </file>
@@ -5407,4 +5417,105 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>115</v>
+      </c>
+      <c r="D2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>180</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>76</v>
+      </c>
+      <c r="D4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>75</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>130</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>